<commit_message>
v2.6: feature - logger
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -489,7 +489,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003732526315901092</v>
+        <v>0.0003646568754914321</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -497,7 +497,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004199092105388729</v>
+        <v>0.0004112749419605073</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -505,7 +505,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.003086756848178432</v>
+        <v>0.003042605804881637</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -513,7 +513,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>9.649428828039756E-05</v>
+        <v>9.427208997079636E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -521,7 +521,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4.241507177160332E-06</v>
+        <v>4.143828130584455E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -529,7 +529,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.802640550293141E-05</v>
+        <v>1.761126955498394E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -537,7 +537,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6.362260765740498E-06</v>
+        <v>6.215742195876684E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -545,7 +545,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001845055622064744</v>
+        <v>0.0001812924807130699</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -553,7 +553,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>4.665657894876365E-05</v>
+        <v>4.558210943642901E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -561,7 +561,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>5.938110048024465E-05</v>
+        <v>5.801359382818238E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -577,7 +577,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>3.181130382870249E-06</v>
+        <v>3.107871097938342E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -585,7 +585,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>1.90867822972215E-05</v>
+        <v>1.864722658763005E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -593,7 +593,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002387968540741267</v>
+        <v>0.002353694378171971</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -601,7 +601,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001747500956990057</v>
+        <v>0.001739371857812825</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -609,7 +609,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>1.060376794290083E-06</v>
+        <v>1.035957032646114E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -617,7 +617,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0006065355263339275</v>
+        <v>0.0005936033797062233</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -625,7 +625,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>4.241507177160332E-06</v>
+        <v>4.143828130584455E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -633,7 +633,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>4.241507177160332E-06</v>
+        <v>4.143828130584455E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -641,7 +641,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>0.0001155810705776191</v>
+        <v>0.0001129193165584264</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -649,7 +649,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0002672149521611009</v>
+        <v>0.0002610611722268207</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -657,7 +657,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0001876866925893447</v>
+        <v>0.0001833643947783622</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -665,7 +665,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>6.25622308631149E-05</v>
+        <v>7.873273448110466E-05</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -673,7 +673,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2.120753588580166E-05</v>
+        <v>2.071914065292228E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -681,7 +681,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.00102008247610706</v>
+        <v>0.001033885118580822</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -689,7 +689,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.378489832577108E-05</v>
+        <v>1.45033984570456E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -697,7 +697,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1.90867822972215E-05</v>
+        <v>1.864722658763005E-05</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -705,7 +705,7 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>1.060376794290083E-06</v>
+        <v>1.035957032646114E-06</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -713,7 +713,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003603160346997702</v>
+        <v>0.00363620918458786</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -721,7 +721,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>7.740750598317607E-05</v>
+        <v>8.080464854639689E-05</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -729,7 +729,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0005153431220249803</v>
+        <v>0.0005625246687268399</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -737,7 +737,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.002824843779988781</v>
+        <v>0.002903787562507058</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.6: fix - 2026/05/14
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -567,7 +567,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003948469526065792</v>
+        <v>0.0003804331921689291</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -575,7 +575,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004148839621418384</v>
+        <v>0.0004107424300065635</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -583,7 +583,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.003214172058979527</v>
+        <v>0.003088406821041718</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -591,7 +591,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4.478860954940302E-05</v>
+        <v>3.971555302862446E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -599,7 +599,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4.714590478884528E-06</v>
+        <v>4.180584529328891E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -607,7 +607,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>2.121565715498037E-05</v>
+        <v>1.881263038198001E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -615,7 +615,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>7.071885718326792E-06</v>
+        <v>7.316022926325559E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -623,7 +623,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001390804191270936</v>
+        <v>0.0001233272436152023</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -631,7 +631,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>4.125266669023962E-05</v>
+        <v>3.65801146316278E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -639,7 +639,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>4.243131430996075E-05</v>
+        <v>3.762526076396002E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -655,7 +655,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>2.357295239442264E-06</v>
+        <v>3.135438396996668E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -663,7 +663,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.30021333521917E-05</v>
+        <v>4.389613755795335E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -671,7 +671,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.00224885965842792</v>
+        <v>0.00218644570883901</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -679,7 +679,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001875228362976321</v>
+        <v>0.001897985376315316</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -687,7 +687,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.357295239442264E-06</v>
+        <v>2.090292264664445E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -695,7 +695,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001815117334370543</v>
+        <v>0.0001609525043791623</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -703,7 +703,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>1.178647619721132E-06</v>
+        <v>2.090292264664445E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -711,7 +711,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>3.535942859163396E-06</v>
+        <v>6.270876793993336E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -719,7 +719,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>7.307615242271019E-05</v>
+        <v>6.688935246926225E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -727,7 +727,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0003088056763669366</v>
+        <v>0.0004180584529328891</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -735,7 +735,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0002039060382117558</v>
+        <v>0.0001891714499521323</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -743,7 +743,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>9.429180957769055E-05</v>
+        <v>8.465683671891004E-05</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -751,7 +751,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2.59302476338649E-05</v>
+        <v>2.29932149113089E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -759,7 +759,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.0008792711243119644</v>
+        <v>0.0007922207683078248</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -767,7 +767,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.650106667609585E-05</v>
+        <v>1.567719198498334E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -775,7 +775,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1.296512381693245E-05</v>
+        <v>1.149660745565445E-05</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -791,7 +791,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.0040604410499393</v>
+        <v>0.0038273251366006</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -799,7 +799,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>9.429180957769055E-05</v>
+        <v>8.674712898357449E-05</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -807,7 +807,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0007272255813679385</v>
+        <v>0.0006657580862956258</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -815,7 +815,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.003253067430430324</v>
+        <v>0.00292013829373623</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -839,7 +839,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -847,7 +847,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.532241905637471E-05</v>
+        <v>1.358689972031889E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -855,7 +855,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>5.89323809860566E-06</v>
+        <v>5.225730661661113E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -871,7 +871,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.535942859163396E-05</v>
+        <v>3.135438396996668E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -887,7 +887,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.0002003700953525924</v>
+        <v>0.0001797651347611423</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -895,7 +895,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -903,7 +903,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -911,7 +911,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>7.071885718326792E-06</v>
+        <v>6.270876793993336E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -919,7 +919,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>2.710889525358604E-05</v>
+        <v>2.508350717597334E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -927,7 +927,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -935,7 +935,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.001004207772002405</v>
+        <v>0.0008956902354087149</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -943,7 +943,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>7.071885718326792E-06</v>
+        <v>6.270876793993336E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -959,7 +959,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0004620298669306837</v>
+        <v>0.0004117875761388958</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -967,7 +967,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>4.478860954940302E-05</v>
+        <v>4.076069916095669E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -975,7 +975,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>2.357295239442264E-06</v>
+        <v>2.090292264664445E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -983,7 +983,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -991,7 +991,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>5.89323809860566E-06</v>
+        <v>5.225730661661113E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -999,7 +999,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>3.535942859163396E-06</v>
+        <v>3.135438396996668E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1007,7 +1007,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.001015994248199616</v>
+        <v>0.0009124125735260304</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1015,7 +1015,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>2.239430477470151E-05</v>
+        <v>1.985777651431223E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1023,7 +1023,7 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>1.178647619721132E-06</v>
+        <v>1.045146132332223E-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.6: fix - xlsx to csv
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>defect_desc</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>青/粉斑Mura</t>
+  </si>
+  <si>
+    <t>灰阶局部暗斑</t>
   </si>
 </sst>
 </file>
@@ -551,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B59"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -567,7 +570,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003804331921689291</v>
+        <v>0.0003958763725919217</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -575,7 +578,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004107424300065635</v>
+        <v>0.000399947080793381</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -583,7 +586,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.003088406821041718</v>
+        <v>0.003011306392029553</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -591,7 +594,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3.971555302862446E-05</v>
+        <v>4.579546726641767E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -599,7 +602,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4.180584529328891E-06</v>
+        <v>4.070708201459349E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -607,7 +610,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.881263038198001E-05</v>
+        <v>1.831818690656707E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -615,7 +618,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>7.316022926325559E-06</v>
+        <v>7.123739352553861E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -623,7 +626,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001233272436152023</v>
+        <v>0.0001282273083459695</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -631,7 +634,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>3.65801146316278E-05</v>
+        <v>3.56186967627693E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -639,7 +642,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.762526076396002E-05</v>
+        <v>3.663637381313414E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -655,7 +658,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>3.135438396996668E-06</v>
+        <v>3.053031151094512E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -663,7 +666,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4.389613755795335E-05</v>
+        <v>4.274243611532316E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -671,7 +674,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.00218644570883901</v>
+        <v>0.002134068774615064</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -679,7 +682,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001897985376315316</v>
+        <v>0.001851154554613639</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -687,7 +690,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.090292264664445E-06</v>
+        <v>2.035354100729674E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -695,7 +698,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001609525043791623</v>
+        <v>0.0001648636821591036</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -703,7 +706,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>2.090292264664445E-06</v>
+        <v>2.035354100729674E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -711,7 +714,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>6.270876793993336E-06</v>
+        <v>6.106062302189024E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -719,7 +722,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>6.688935246926225E-05</v>
+        <v>7.327274762626828E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -727,7 +730,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0004180584529328891</v>
+        <v>0.0004528662874123526</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -735,7 +738,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0001891714499521323</v>
+        <v>0.0001943763166196839</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -743,7 +746,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>8.465683671891004E-05</v>
+        <v>0.0001170328607919563</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -751,7 +754,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2.29932149113089E-05</v>
+        <v>2.238889510802642E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -759,7 +762,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.0007922207683078248</v>
+        <v>0.0009087856059757997</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -767,7 +770,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.567719198498334E-05</v>
+        <v>1.526515575547256E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -775,7 +778,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1.149660745565445E-05</v>
+        <v>1.119444755401321E-05</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -791,7 +794,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.0038273251366006</v>
+        <v>0.00399947080793381</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -799,7 +802,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>8.674712898357449E-05</v>
+        <v>8.752022633137601E-05</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -807,7 +810,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0006657580862956258</v>
+        <v>0.0006686138220896981</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -815,7 +818,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.00292013829373623</v>
+        <v>0.002942104352604745</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -839,7 +842,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -847,7 +850,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.358689972031889E-05</v>
+        <v>1.424747870510772E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -855,7 +858,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>5.225730661661113E-06</v>
+        <v>5.088385251824186E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -863,7 +866,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>9.711915451948841E-07</v>
+        <v>2.035354100729674E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -871,7 +874,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.135438396996668E-05</v>
+        <v>3.053031151094512E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -887,7 +890,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.0001797651347611423</v>
+        <v>0.000181146514964941</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -895,7 +898,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -903,7 +906,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -911,7 +914,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>6.270876793993336E-06</v>
+        <v>6.106062302189024E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -919,7 +922,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>2.508350717597334E-05</v>
+        <v>2.544192625912093E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -927,7 +930,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -935,7 +938,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0008956902354087149</v>
+        <v>0.0008802906485655842</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -943,7 +946,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>6.270876793993336E-06</v>
+        <v>7.123739352553861E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -959,7 +962,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0004117875761388958</v>
+        <v>0.0004223359759014075</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -967,7 +970,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>4.076069916095669E-05</v>
+        <v>3.968940496422865E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -975,7 +978,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>2.090292264664445E-06</v>
+        <v>2.035354100729674E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -983,7 +986,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -991,7 +994,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>5.225730661661113E-06</v>
+        <v>6.106062302189024E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -999,7 +1002,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>3.135438396996668E-06</v>
+        <v>4.070708201459349E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1007,7 +1010,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.0009124125735260304</v>
+        <v>0.0009260861158320019</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1015,7 +1018,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.985777651431223E-05</v>
+        <v>1.933586395693191E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1023,7 +1026,15 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>1.045146132332223E-06</v>
+        <v>1.017677050364837E-06</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60">
+        <v>1.017677050364837E-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V2.8: module - 关键备件
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -570,7 +570,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003958763725919217</v>
+        <v>0.0003958759697180325</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -578,7 +578,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.000399947080793381</v>
+        <v>0.0003999466737768298</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -586,7 +586,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.003011306392029553</v>
+        <v>0.003011303327495265</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -594,7 +594,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4.579546726641767E-05</v>
+        <v>4.579542066146906E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -602,7 +602,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4.070708201459349E-06</v>
+        <v>4.070704058797249E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -610,7 +610,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.831818690656707E-05</v>
+        <v>1.831816826458762E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -618,7 +618,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>7.123739352553861E-06</v>
+        <v>7.123732102895187E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -626,7 +626,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001282273083459695</v>
+        <v>0.0001282271778521133</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -634,7 +634,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>3.56186967627693E-05</v>
+        <v>3.561866051447594E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -642,7 +642,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.663637381313414E-05</v>
+        <v>3.663633652917525E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -658,7 +658,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>3.053031151094512E-06</v>
+        <v>3.053028044097937E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -666,7 +666,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4.274243611532316E-05</v>
+        <v>4.274239261737112E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -674,7 +674,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002134068774615064</v>
+        <v>0.002134066602824458</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -682,7 +682,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001851154554613639</v>
+        <v>0.001851152670738049</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -690,7 +690,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.035354100729674E-06</v>
+        <v>2.035352029398625E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -698,7 +698,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001648636821591036</v>
+        <v>0.0001648635143812886</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -706,7 +706,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>2.035354100729674E-06</v>
+        <v>2.035352029398625E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -714,7 +714,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>6.106062302189024E-06</v>
+        <v>6.106056088195874E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -722,7 +722,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>7.327274762626828E-05</v>
+        <v>7.327267305835049E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -730,7 +730,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0004528662874123526</v>
+        <v>0.000452865826541194</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -738,7 +738,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0001943763166196839</v>
+        <v>0.0001943761188075687</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -746,7 +746,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001170328607919563</v>
+        <v>0.0001170327416904209</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -754,7 +754,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2.238889510802642E-05</v>
+        <v>2.238887232338487E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -762,7 +762,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.0009087856059757997</v>
+        <v>0.000908784681126486</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -770,7 +770,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.526515575547256E-05</v>
+        <v>1.526514022048969E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -778,7 +778,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1.119444755401321E-05</v>
+        <v>1.119443616169244E-05</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -794,7 +794,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.00399947080793381</v>
+        <v>0.003999466737768298</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -802,7 +802,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>8.752022633137601E-05</v>
+        <v>8.752013726414087E-05</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -810,7 +810,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0006686138220896981</v>
+        <v>0.0006686131416574482</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -818,7 +818,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.002942104352604745</v>
+        <v>0.002942101358495712</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -842,7 +842,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -850,7 +850,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.424747870510772E-05</v>
+        <v>1.424746420579037E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -858,7 +858,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>5.088385251824186E-06</v>
+        <v>5.088380073496562E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -866,7 +866,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>2.035354100729674E-06</v>
+        <v>2.035352029398625E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -874,7 +874,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.053031151094512E-05</v>
+        <v>3.053028044097937E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -890,7 +890,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.000181146514964941</v>
+        <v>0.0001811463306164776</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -898,7 +898,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -906,7 +906,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -914,7 +914,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>6.106062302189024E-06</v>
+        <v>6.106056088195874E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -922,7 +922,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>2.544192625912093E-05</v>
+        <v>2.544190036748281E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -930,7 +930,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -938,7 +938,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0008802906485655842</v>
+        <v>0.0008802897527149052</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -946,7 +946,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>7.123739352553861E-06</v>
+        <v>7.123732102895187E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -962,7 +962,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0004223359759014075</v>
+        <v>0.0004223355461002146</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -970,7 +970,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.968940496422865E-05</v>
+        <v>3.968936457327318E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -978,7 +978,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>2.035354100729674E-06</v>
+        <v>2.035352029398625E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -986,7 +986,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -994,7 +994,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>6.106062302189024E-06</v>
+        <v>6.106056088195874E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1002,7 +1002,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>4.070708201459349E-06</v>
+        <v>4.070704058797249E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1010,7 +1010,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.0009260861158320019</v>
+        <v>0.0009260851733763742</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1018,7 +1018,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.933586395693191E-05</v>
+        <v>1.933584427928693E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1026,7 +1026,7 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1034,7 +1034,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>1.017677050364837E-06</v>
+        <v>1.017676014699312E-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.8: fix - 2026/05/29
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -576,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003807366343228438</v>
+        <v>0.0003615637862593557</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -584,7 +584,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004119587729005714</v>
+        <v>0.0004134336965244109</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -592,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.003229756779540479</v>
+        <v>0.002564509386928172</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -600,7 +600,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>8.239175458011427E-05</v>
+        <v>7.475369420552079E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>3.469126508636391E-06</v>
+        <v>6.102342384124146E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -616,7 +616,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.821291417034105E-05</v>
+        <v>1.906981995038796E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6.938253017272781E-06</v>
+        <v>6.102342384124146E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -632,7 +632,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001517742847528421</v>
+        <v>0.0001426422532289019</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>3.122213857772751E-05</v>
+        <v>2.974891912260521E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.38239834592048E-05</v>
+        <v>3.280009031466728E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>7.805534644431878E-06</v>
+        <v>7.627927980155183E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.64258283406821E-05</v>
+        <v>3.813963990077591E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002324314760786381</v>
+        <v>0.002266257402904105</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001954852787616606</v>
+        <v>0.00189096334628047</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>1.734563254318195E-06</v>
+        <v>2.288378394046555E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001621816642787513</v>
+        <v>0.0001525585596031036</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -712,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>5.203689762954586E-06</v>
+        <v>4.57675678809311E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -720,7 +720,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>6.070971390113683E-06</v>
+        <v>5.339549586108628E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -728,7 +728,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>8.325903620727337E-05</v>
+        <v>7.475369420552079E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -736,7 +736,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0003885421689672757</v>
+        <v>0.0003844475701998212</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -744,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0001916692396021606</v>
+        <v>0.0002799449568716952</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001734563254318195</v>
+        <v>0.0001731539651495226</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -760,7 +760,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2.081475905181834E-05</v>
+        <v>1.906981995038796E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -768,7 +768,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.001164759225274668</v>
+        <v>0.001196821900086348</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.300922440738646E-05</v>
+        <v>1.601864875832588E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -784,7 +784,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>9.540097898750074E-06</v>
+        <v>9.153513576186219E-06</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -800,7 +800,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003822977412517302</v>
+        <v>0.003862782729150584</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -808,7 +808,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>9.193185247886435E-05</v>
+        <v>0.0001189956764904208</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -816,7 +816,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0008039700683764835</v>
+        <v>0.0008283929786448528</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -824,7 +824,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.00298865248719025</v>
+        <v>0.002985571011432739</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -848,7 +848,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -856,7 +856,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.300922440738646E-05</v>
+        <v>1.296747756626381E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -864,7 +864,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>4.336408135795488E-06</v>
+        <v>3.813963990077591E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -872,7 +872,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>1.734563254318195E-06</v>
+        <v>1.525585596031036E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -880,7 +880,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.035485695056842E-05</v>
+        <v>3.051171192062073E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -896,7 +896,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.0001855982682120469</v>
+        <v>0.000169340001159445</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -904,7 +904,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>8.672816271590977E-07</v>
+        <v>2.288378394046555E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -912,7 +912,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -920,7 +920,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>6.938253017272781E-06</v>
+        <v>7.627927980155183E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>2.168204067897744E-05</v>
+        <v>1.906981995038796E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -936,7 +936,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -944,7 +944,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0008299885171912564</v>
+        <v>0.0006010807248362284</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -952,7 +952,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>8.672816271590975E-06</v>
+        <v>9.153513576186219E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -968,7 +968,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0004076223647647759</v>
+        <v>0.000397415047766085</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -976,7 +976,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.64258283406821E-05</v>
+        <v>3.661405430474488E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -984,7 +984,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>1.734563254318195E-06</v>
+        <v>1.525585596031036E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -992,7 +992,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>8.672816271590977E-07</v>
+        <v>2.288378394046555E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>6.070971390113683E-06</v>
+        <v>7.627927980155183E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>3.469126508636391E-06</v>
+        <v>4.57675678809311E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.001017321348657622</v>
+        <v>0.0008390720778170701</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.821291417034105E-05</v>
+        <v>1.67814415563414E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1032,7 +1032,7 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>61</v>
       </c>
       <c r="B61">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>62</v>
       </c>
       <c r="B62">
-        <v>8.672816271590977E-07</v>
+        <v>7.627927980155182E-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.8: feat - parts
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -576,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003615637862593557</v>
+        <v>0.0003572683084996833</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -584,7 +584,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004134336965244109</v>
+        <v>0.000406805510938715</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -592,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.002564509386928172</v>
+        <v>0.002523395069697343</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -600,7 +600,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>7.475369420552079E-05</v>
+        <v>7.505636733186623E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>6.102342384124146E-06</v>
+        <v>6.004509386549298E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -616,7 +616,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.906981995038796E-05</v>
+        <v>1.876409183296656E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6.102342384124146E-06</v>
+        <v>6.004509386549298E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -632,7 +632,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001426422532289019</v>
+        <v>0.0001411059705839085</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>2.974891912260521E-05</v>
+        <v>2.927198325942783E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.280009031466728E-05</v>
+        <v>3.227423795270248E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>7.627927980155183E-06</v>
+        <v>7.505636733186623E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.813963990077591E-05</v>
+        <v>3.752818366593311E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002266257402904105</v>
+        <v>0.002230675237103064</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.00189096334628047</v>
+        <v>0.001860647346156964</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.288378394046555E-06</v>
+        <v>2.251691019955987E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001525585596031036</v>
+        <v>0.0001523644256836885</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -712,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>4.57675678809311E-06</v>
+        <v>4.503382039911974E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -720,7 +720,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>5.339549586108628E-06</v>
+        <v>5.253945713230636E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -728,7 +728,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>7.475369420552079E-05</v>
+        <v>7.655749467850356E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -736,7 +736,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0003844475701998212</v>
+        <v>0.0003782840913526058</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -744,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0002799449568716952</v>
+        <v>0.000286715323207729</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001731539651495226</v>
+        <v>0.0001703779538433364</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -760,7 +760,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>1.906981995038796E-05</v>
+        <v>1.876409183296656E-05</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -768,7 +768,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.001196821900086348</v>
+        <v>0.001209158077716365</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.601864875832588E-05</v>
+        <v>1.651240081301057E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -784,7 +784,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>9.153513576186219E-06</v>
+        <v>9.006764079823948E-06</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -800,7 +800,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003862782729150584</v>
+        <v>0.003890171518810627</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -808,7 +808,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>0.0001189956764904208</v>
+        <v>0.0001208407514043046</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -816,7 +816,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0008283929786448528</v>
+        <v>0.0008563931512565937</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -824,7 +824,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.002985571011432739</v>
+        <v>0.003024771603474209</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -848,7 +848,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -856,7 +856,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.296747756626381E-05</v>
+        <v>1.426070979305458E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -864,7 +864,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>3.813963990077591E-06</v>
+        <v>3.752818366593312E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -872,7 +872,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>1.525585596031036E-06</v>
+        <v>1.501127346637325E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -880,7 +880,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.051171192062073E-05</v>
+        <v>3.002254693274649E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -896,7 +896,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.000169340001159445</v>
+        <v>0.0001703779538433364</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -904,7 +904,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>2.288378394046555E-06</v>
+        <v>2.251691019955987E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -912,7 +912,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -920,7 +920,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>7.627927980155183E-06</v>
+        <v>7.505636733186623E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>1.906981995038796E-05</v>
+        <v>1.876409183296656E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -936,7 +936,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -944,7 +944,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0006010807248362284</v>
+        <v>0.0005914441745751059</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -952,7 +952,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>9.153513576186219E-06</v>
+        <v>9.006764079823948E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -968,7 +968,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.000397415047766085</v>
+        <v>0.000404553819918759</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -976,7 +976,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.661405430474488E-05</v>
+        <v>3.827874733925178E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -984,7 +984,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>1.525585596031036E-06</v>
+        <v>1.501127346637325E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -992,7 +992,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>2.288378394046555E-06</v>
+        <v>3.002254693274649E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>7.627927980155183E-06</v>
+        <v>7.505636733186623E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>4.57675678809311E-06</v>
+        <v>4.503382039911974E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.0008390720778170701</v>
+        <v>0.0008451346961568137</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.67814415563414E-05</v>
+        <v>1.726296448632923E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1032,7 +1032,7 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>61</v>
       </c>
       <c r="B61">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>62</v>
       </c>
       <c r="B62">
-        <v>7.627927980155182E-07</v>
+        <v>7.505636733186623E-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.8: fix - 2026/06/05
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -576,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003572683084996833</v>
+        <v>0.0003066748970869816</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -584,7 +584,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.000406805510938715</v>
+        <v>0.0004128315922324753</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -592,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.002523395069697343</v>
+        <v>0.002534392803362415</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -600,7 +600,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>7.505636733186623E-05</v>
+        <v>7.391651365686224E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>6.004509386549298E-06</v>
+        <v>6.290767119732957E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -616,7 +616,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>1.876409183296656E-05</v>
+        <v>2.201768491906535E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6.004509386549298E-06</v>
+        <v>7.077113009699577E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -632,7 +632,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001411059705839085</v>
+        <v>9.672054446589421E-05</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>2.927198325942783E-05</v>
+        <v>2.830845203879831E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.227423795270248E-05</v>
+        <v>3.853094860836436E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>7.505636733186623E-06</v>
+        <v>7.863458899666196E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.752818366593311E-05</v>
+        <v>3.853094860836436E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002230675237103064</v>
+        <v>0.002247376553524599</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001860647346156964</v>
+        <v>0.001894307248929587</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.251691019955987E-06</v>
+        <v>5.504421229766337E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.0001523644256836885</v>
+        <v>9.907958213579407E-05</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -712,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>4.503382039911974E-06</v>
+        <v>5.504421229766337E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -720,7 +720,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>5.253945713230636E-06</v>
+        <v>4.718075339799718E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -728,7 +728,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>7.655749467850356E-05</v>
+        <v>5.504421229766337E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -736,7 +736,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0003782840913526058</v>
+        <v>0.0003184700854364809</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -744,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.000286715323207729</v>
+        <v>0.0002374764587699191</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001703779538433364</v>
+        <v>0.0001863639759220888</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -760,7 +760,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>1.876409183296656E-05</v>
+        <v>7.077113009699577E-06</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -768,7 +768,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.001209158077716365</v>
+        <v>0.001162219225370664</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1.651240081301057E-05</v>
+        <v>2.594941436889845E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -784,7 +784,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>9.006764079823948E-06</v>
+        <v>7.863458899666196E-06</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -800,7 +800,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003890171518810627</v>
+        <v>0.003663585501354481</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -808,7 +808,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>0.0001208407514043046</v>
+        <v>0.0001360378389642252</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -816,7 +816,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0008563931512565937</v>
+        <v>0.0009349652631703107</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -824,7 +824,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.003024771603474209</v>
+        <v>0.002752996960773135</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -848,7 +848,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>7.505636733186623E-07</v>
+        <v>1.572691779933239E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -856,7 +856,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.426070979305458E-05</v>
+        <v>1.336788012943253E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -864,7 +864,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>3.752818366593312E-06</v>
+        <v>3.145383559866478E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -872,7 +872,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>1.501127346637325E-06</v>
+        <v>1.572691779933239E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -880,7 +880,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.002254693274649E-05</v>
+        <v>3.695825682843112E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -896,7 +896,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.0001703779538433364</v>
+        <v>0.0001533374485434908</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -904,7 +904,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>2.251691019955987E-06</v>
+        <v>2.359037669899859E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -912,7 +912,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>7.505636733186623E-07</v>
+        <v>7.863458899666196E-07</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -920,7 +920,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>7.505636733186623E-06</v>
+        <v>7.863458899666196E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>1.876409183296656E-05</v>
+        <v>1.729960957926563E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -936,7 +936,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>7.505636733186623E-07</v>
+        <v>7.863458899666196E-07</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -944,7 +944,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0005914441745751059</v>
+        <v>0.0003349833491257799</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -952,7 +952,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>9.006764079823948E-06</v>
+        <v>9.436150679599436E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -968,7 +968,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.000404553819918759</v>
+        <v>0.0003978910203231095</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -976,7 +976,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.827874733925178E-05</v>
+        <v>3.459921915853126E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -984,7 +984,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>1.501127346637325E-06</v>
+        <v>1.497346701644686E-06</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -992,7 +992,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>3.002254693274649E-06</v>
+        <v>3.145383559866478E-06</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>7.505636733186623E-06</v>
+        <v>7.863458899666196E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>4.503382039911974E-06</v>
+        <v>3.931729449833098E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.0008451346961568137</v>
+        <v>0.001080439252814135</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.726296448632923E-05</v>
+        <v>1.729960957926563E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1032,7 +1032,7 @@
         <v>59</v>
       </c>
       <c r="B59">
-        <v>7.505636733186623E-07</v>
+        <v>7.486733508223428E-07</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>7.505636733186623E-07</v>
+        <v>7.863458899666196E-07</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>61</v>
       </c>
       <c r="B61">
-        <v>7.505636733186623E-07</v>
+        <v>7.863458899666196E-07</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>62</v>
       </c>
       <c r="B62">
-        <v>7.505636733186623E-07</v>
+        <v>7.863458899666196E-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.8: refactor - Harness
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -576,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.0003066748970869816</v>
+        <v>0.000303812118727847</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -584,7 +584,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.0004128315922324753</v>
+        <v>0.000418172235981413</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -592,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.002534392803362415</v>
+        <v>0.00260065929296513</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -600,7 +600,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>7.391651365686224E-05</v>
+        <v>7.509188422071503E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>6.290767119732957E-06</v>
+        <v>5.511330951979085E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -616,7 +616,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>2.201768491906535E-05</v>
+        <v>2.066749106992157E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>7.077113009699577E-06</v>
+        <v>6.20024732097647E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -632,7 +632,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>9.672054446589421E-05</v>
+        <v>0.0001178046990985529</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>2.830845203879831E-05</v>
+        <v>2.548990565290327E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.853094860836436E-05</v>
+        <v>3.513473481886666E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>7.863458899666196E-06</v>
+        <v>8.266996427968628E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.853094860836436E-05</v>
+        <v>3.375690208087189E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002247376553524599</v>
+        <v>0.002370561225720004</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001894307248929587</v>
+        <v>0.001928276916823682</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>5.504421229766337E-06</v>
+        <v>4.822414582981699E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>9.907958213579407E-05</v>
+        <v>8.680346249367057E-05</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -712,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>5.504421229766337E-06</v>
+        <v>5.511330951979085E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -720,7 +720,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>4.718075339799718E-06</v>
+        <v>4.822414582981699E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -728,7 +728,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>5.504421229766337E-05</v>
+        <v>5.373547678179607E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -736,7 +736,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0003184700854364809</v>
+        <v>0.0002845224603959202</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -744,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0002374764587699191</v>
+        <v>0.0002080527434372104</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001863639759220888</v>
+        <v>0.0001667177612973673</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -760,7 +760,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>7.077113009699577E-06</v>
+        <v>6.20024732097647E-06</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -768,7 +768,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.001162219225370664</v>
+        <v>0.001104332939502809</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>2.594941436889845E-05</v>
+        <v>2.273424017691372E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -784,7 +784,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>7.863458899666196E-06</v>
+        <v>6.889163689973856E-06</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -800,7 +800,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003663585501354481</v>
+        <v>0.003525185060159622</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -808,7 +808,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>0.0001360378389642252</v>
+        <v>0.0001219381973125373</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -816,7 +816,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.0009349652631703107</v>
+        <v>0.001151868168963629</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -824,7 +824,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.002752996960773135</v>
+        <v>0.002563457809039272</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -848,7 +848,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1.572691779933239E-06</v>
+        <v>1.377832737994771E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -856,7 +856,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.336788012943253E-05</v>
+        <v>1.171157827295555E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -864,7 +864,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>3.145383559866478E-06</v>
+        <v>2.755665475989542E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -872,7 +872,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>1.572691779933239E-06</v>
+        <v>1.377832737994771E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -880,7 +880,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.695825682843112E-05</v>
+        <v>3.926823303285097E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -896,7 +896,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.0001533374485434908</v>
+        <v>0.000141227855644464</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -904,7 +904,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>2.359037669899859E-06</v>
+        <v>2.066749106992157E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -912,7 +912,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>7.863458899666196E-07</v>
+        <v>6.889163689973856E-07</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -920,7 +920,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>7.863458899666196E-06</v>
+        <v>9.644829165963398E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>1.729960957926563E-05</v>
+        <v>1.515616011794248E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -936,7 +936,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>7.863458899666196E-07</v>
+        <v>6.889163689973856E-07</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -944,7 +944,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0003349833491257799</v>
+        <v>0.0002962340386688758</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -952,7 +952,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>9.436150679599436E-06</v>
+        <v>8.955912796966012E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -968,7 +968,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0003978910203231095</v>
+        <v>0.0003768372538415699</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -976,7 +976,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.459921915853126E-05</v>
+        <v>3.720148392585882E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -992,7 +992,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>3.145383559866478E-06</v>
+        <v>2.135640743891895E-05</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>7.863458899666196E-06</v>
+        <v>8.955912796966012E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>3.931729449833098E-06</v>
+        <v>3.444581844986928E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.001080439252814135</v>
+        <v>0.001161512998129592</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.729960957926563E-05</v>
+        <v>1.515616011794248E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>7.863458899666196E-07</v>
+        <v>6.889163689973856E-07</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>61</v>
       </c>
       <c r="B61">
-        <v>7.863458899666196E-07</v>
+        <v>6.889163689973856E-07</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>62</v>
       </c>
       <c r="B62">
-        <v>7.863458899666196E-07</v>
+        <v>6.889163689973856E-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.8: fix - refresh and cache
</commit_message>
<xml_diff>
--- a/resources/M626/M626_codebaseline.xlsx
+++ b/resources/M626/M626_codebaseline.xlsx
@@ -576,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.000303812118727847</v>
+        <v>0.0003757436593257489</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -584,7 +584,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.000418172235981413</v>
+        <v>0.0003979229725498382</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -592,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.00260065929296513</v>
+        <v>0.002515395052708486</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -600,7 +600,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>7.509188422071503E-05</v>
+        <v>7.175660160734788E-05</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>5.511330951979085E-06</v>
+        <v>5.218661935079846E-06</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -616,7 +616,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>2.066749106992157E-05</v>
+        <v>2.02223149984344E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6.20024732097647E-06</v>
+        <v>5.870994676964826E-06</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -632,7 +632,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.0001178046990985529</v>
+        <v>0.0001167675607974115</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -640,7 +640,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>2.548990565290327E-05</v>
+        <v>2.413631144974428E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -648,7 +648,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3.513473481886666E-05</v>
+        <v>3.326896983613402E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>8.266996427968628E-06</v>
+        <v>7.827992902619769E-06</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3.375690208087189E-05</v>
+        <v>3.196430435236405E-05</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.002370561225720004</v>
+        <v>0.002266203945308423</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -688,7 +688,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.001928276916823682</v>
+        <v>0.00186501930904916</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>4.822414582981699E-06</v>
+        <v>4.566329193194865E-06</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>8.680346249367057E-05</v>
+        <v>8.219392547750757E-05</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -712,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>5.511330951979085E-06</v>
+        <v>5.870994676964826E-06</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -720,7 +720,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>4.822414582981699E-06</v>
+        <v>4.566329193194865E-06</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -728,7 +728,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>5.373547678179607E-05</v>
+        <v>5.349128483456841E-05</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -736,7 +736,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.0002845224603959202</v>
+        <v>0.000272675086107922</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -744,7 +744,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.0002080527434372104</v>
+        <v>0.0001970044880492642</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -752,7 +752,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0.0001667177612973673</v>
+        <v>0.0001617785199874752</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -760,7 +760,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>6.20024732097647E-06</v>
+        <v>5.870994676964826E-06</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -768,7 +768,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0.001104332939502809</v>
+        <v>0.001061997703788748</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -776,7 +776,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>2.273424017691372E-05</v>
+        <v>2.152698048220436E-05</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -784,7 +784,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>6.889163689973856E-06</v>
+        <v>6.523327418849807E-06</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -800,7 +800,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0.003525185060159622</v>
+        <v>0.00354803778311241</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -808,7 +808,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>0.0001219381973125373</v>
+        <v>0.0001206815572487214</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -816,7 +816,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0.001151868168963629</v>
+        <v>0.001102442333785617</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -824,7 +824,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0.002563457809039272</v>
+        <v>0.002465817764325227</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -848,7 +848,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1.377832737994771E-06</v>
+        <v>1.304665483769961E-06</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -856,7 +856,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1.171157827295555E-05</v>
+        <v>1.239432209581463E-05</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -864,7 +864,7 @@
         <v>38</v>
       </c>
       <c r="B38">
-        <v>2.755665475989542E-06</v>
+        <v>2.609330967539923E-06</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -872,7 +872,7 @@
         <v>39</v>
       </c>
       <c r="B39">
-        <v>1.377832737994771E-06</v>
+        <v>1.304665483769961E-06</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -880,7 +880,7 @@
         <v>40</v>
       </c>
       <c r="B40">
-        <v>3.926823303285097E-05</v>
+        <v>3.848763177121386E-05</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -896,7 +896,7 @@
         <v>42</v>
       </c>
       <c r="B42">
-        <v>0.000141227855644464</v>
+        <v>0.0001409038722471558</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -904,7 +904,7 @@
         <v>43</v>
       </c>
       <c r="B43">
-        <v>2.066749106992157E-06</v>
+        <v>1.956998225654942E-06</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -912,7 +912,7 @@
         <v>44</v>
       </c>
       <c r="B44">
-        <v>6.889163689973856E-07</v>
+        <v>6.523327418849807E-07</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -920,7 +920,7 @@
         <v>45</v>
       </c>
       <c r="B45">
-        <v>9.644829165963398E-06</v>
+        <v>9.13265838638973E-06</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
       <c r="B46">
-        <v>1.515616011794248E-05</v>
+        <v>1.435132032146958E-05</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -936,7 +936,7 @@
         <v>47</v>
       </c>
       <c r="B47">
-        <v>6.889163689973856E-07</v>
+        <v>1.956998225654942E-06</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -944,7 +944,7 @@
         <v>48</v>
       </c>
       <c r="B48">
-        <v>0.0002962340386688758</v>
+        <v>0.0002805030790105417</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -952,7 +952,7 @@
         <v>49</v>
       </c>
       <c r="B49">
-        <v>8.955912796966012E-06</v>
+        <v>8.48032564450475E-06</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -968,7 +968,7 @@
         <v>51</v>
       </c>
       <c r="B51">
-        <v>0.0003768372538415699</v>
+        <v>0.0003659586681974742</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -976,7 +976,7 @@
         <v>52</v>
       </c>
       <c r="B52">
-        <v>3.720148392585882E-05</v>
+        <v>3.522596806178896E-05</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -984,7 +984,7 @@
         <v>53</v>
       </c>
       <c r="B53">
-        <v>1.497346701644686E-06</v>
+        <v>6.523327418849807E-07</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -992,7 +992,7 @@
         <v>54</v>
       </c>
       <c r="B54">
-        <v>2.135640743891895E-05</v>
+        <v>2.152698048220436E-05</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -1000,7 +1000,7 @@
         <v>55</v>
       </c>
       <c r="B55">
-        <v>8.955912796966012E-06</v>
+        <v>8.48032564450475E-06</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -1008,7 +1008,7 @@
         <v>56</v>
       </c>
       <c r="B56">
-        <v>3.444581844986928E-06</v>
+        <v>3.261663709424903E-06</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -1016,7 +1016,7 @@
         <v>57</v>
       </c>
       <c r="B57">
-        <v>0.001161512998129592</v>
+        <v>0.001122664648784052</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -1024,7 +1024,7 @@
         <v>58</v>
       </c>
       <c r="B58">
-        <v>1.515616011794248E-05</v>
+        <v>1.435132032146958E-05</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -1040,7 +1040,7 @@
         <v>60</v>
       </c>
       <c r="B60">
-        <v>6.889163689973856E-07</v>
+        <v>6.523327418849807E-07</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -1048,7 +1048,7 @@
         <v>61</v>
       </c>
       <c r="B61">
-        <v>6.889163689973856E-07</v>
+        <v>6.523327418849807E-07</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -1056,7 +1056,7 @@
         <v>62</v>
       </c>
       <c r="B62">
-        <v>6.889163689973856E-07</v>
+        <v>6.523327418849807E-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>